<commit_message>
feat: home-screen widgets, richer notifications, session telemetry
- Android home widgets: medium 4-stat glance + 1x1 New Sale & Vision AI
- iOS WidgetKit source (KiranaWidget) + Mac setup runbook
- Notifications: per-category channels, BigText + action buttons,
  route+tab+subtab deep-links (shared by widgets)
- Auth: device telemetry headers for the admin Sessions page
- Subscription: fix trial reminder wrongly saying 'expired' when days remain;
  localize the push title
- Local: portrait-only orientation, printer service cleanup, formatting

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Kirana_AI_Feature_Matrix.xlsx
+++ b/Kirana_AI_Feature_Matrix.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bhanuprakash\Documents\FlutterProjects\kirana_ai\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_61D93BA9D2BB45E6850C79515CF100714BFB5D68" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18D04BAD-AA0A-47D5-8BB3-70A6EFD5F194}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="404" uniqueCount="170">
   <si>
     <t>🏪  Kirana AI  ·  Feature Matrix</t>
   </si>
@@ -467,6 +467,72 @@
   </si>
   <si>
     <t>Configurable start/end hour</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  RETAIL INTELLIGENCE (AI)</t>
+  </si>
+  <si>
+    <t>Smart Udhaar reminders (recovery-risk scoring)</t>
+  </si>
+  <si>
+    <t>Intelligence</t>
+  </si>
+  <si>
+    <t>Pro only · ML risk score &amp; recovery likelihood per credit; suggested action + 1-tap WhatsApp reminder</t>
+  </si>
+  <si>
+    <t>AI Price Memory (missing-price fixer)</t>
+  </si>
+  <si>
+    <t>Pro only · Flags unpriced / ₹0 items; one-tap suggested price (your last sold price, else MRP)</t>
+  </si>
+  <si>
+    <t>AI reorder suggestions (velocity-based)</t>
+  </si>
+  <si>
+    <t>Pro only · Days-of-cover &amp; suggested qty with supplier, lead time &amp; reorder cost</t>
+  </si>
+  <si>
+    <t>ML item flags on inventory list</t>
+  </si>
+  <si>
+    <t>Pro only · Fast-moving · Reorder-now · Dead-stock · Stockout-risk · Profit-opportunity tags</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  RETURNS &amp; STOCK OPS</t>
+  </si>
+  <si>
+    <t>Customer returns &amp; exchanges</t>
+  </si>
+  <si>
+    <t>Returns</t>
+  </si>
+  <si>
+    <t>Recorded against a past order; resaleable units restocked, damaged units sent to Return-to-Vendor ledger</t>
+  </si>
+  <si>
+    <t>Near-expiry alerts screen</t>
+  </si>
+  <si>
+    <t>Batch-level items nearing expiry surfaced with counts &amp; quick actions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  LANGUAGES &amp; LOCALIZATION</t>
+  </si>
+  <si>
+    <t>Multi-language (vernacular) UI</t>
+  </si>
+  <si>
+    <t>Localization</t>
+  </si>
+  <si>
+    <t>7 languages: English, Telugu, Hindi, Marathi, Tamil, Kannada, Malayalam · switch anytime in Profile</t>
+  </si>
+  <si>
+    <t>First-run language selection</t>
+  </si>
+  <si>
+    <t>Pick your language on first launch; native-script fonts (Noto) auto-applied so text never renders as boxes</t>
   </si>
 </sst>
 </file>
@@ -691,7 +757,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -714,11 +780,48 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFD1D5DB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD1D5DB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFD1D5DB"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD1D5DB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD1D5DB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD1D5DB"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFD1D5DB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD1D5DB"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -886,8 +989,19 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1191,7 +1305,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F87"/>
+  <dimension ref="A1:F98"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -1202,7 +1316,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="59" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="55"/>
@@ -1245,11 +1359,11 @@
       <c r="A4" s="56" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="55"/>
-      <c r="C4" s="55"/>
-      <c r="D4" s="55"/>
-      <c r="E4" s="55"/>
-      <c r="F4" s="55"/>
+      <c r="B4" s="57"/>
+      <c r="C4" s="57"/>
+      <c r="D4" s="57"/>
+      <c r="E4" s="57"/>
+      <c r="F4" s="58"/>
     </row>
     <row r="5" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4">
@@ -1481,11 +1595,11 @@
       <c r="A17" s="56" t="s">
         <v>29</v>
       </c>
-      <c r="B17" s="55"/>
-      <c r="C17" s="55"/>
-      <c r="D17" s="55"/>
-      <c r="E17" s="55"/>
-      <c r="F17" s="55"/>
+      <c r="B17" s="57"/>
+      <c r="C17" s="57"/>
+      <c r="D17" s="57"/>
+      <c r="E17" s="57"/>
+      <c r="F17" s="58"/>
     </row>
     <row r="18" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4">
@@ -1703,11 +1817,11 @@
       <c r="A29" s="56" t="s">
         <v>49</v>
       </c>
-      <c r="B29" s="55"/>
-      <c r="C29" s="55"/>
-      <c r="D29" s="55"/>
-      <c r="E29" s="55"/>
-      <c r="F29" s="55"/>
+      <c r="B29" s="57"/>
+      <c r="C29" s="57"/>
+      <c r="D29" s="57"/>
+      <c r="E29" s="57"/>
+      <c r="F29" s="58"/>
     </row>
     <row r="30" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="4">
@@ -1853,11 +1967,11 @@
       <c r="A37" s="56" t="s">
         <v>63</v>
       </c>
-      <c r="B37" s="55"/>
-      <c r="C37" s="55"/>
-      <c r="D37" s="55"/>
-      <c r="E37" s="55"/>
-      <c r="F37" s="55"/>
+      <c r="B37" s="57"/>
+      <c r="C37" s="57"/>
+      <c r="D37" s="57"/>
+      <c r="E37" s="57"/>
+      <c r="F37" s="58"/>
     </row>
     <row r="38" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="4">
@@ -1957,11 +2071,11 @@
       <c r="A43" s="56" t="s">
         <v>72</v>
       </c>
-      <c r="B43" s="55"/>
-      <c r="C43" s="55"/>
-      <c r="D43" s="55"/>
-      <c r="E43" s="55"/>
-      <c r="F43" s="55"/>
+      <c r="B43" s="57"/>
+      <c r="C43" s="57"/>
+      <c r="D43" s="57"/>
+      <c r="E43" s="57"/>
+      <c r="F43" s="58"/>
     </row>
     <row r="44" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="4">
@@ -2087,11 +2201,11 @@
       <c r="A50" s="56" t="s">
         <v>82</v>
       </c>
-      <c r="B50" s="55"/>
-      <c r="C50" s="55"/>
-      <c r="D50" s="55"/>
-      <c r="E50" s="55"/>
-      <c r="F50" s="55"/>
+      <c r="B50" s="57"/>
+      <c r="C50" s="57"/>
+      <c r="D50" s="57"/>
+      <c r="E50" s="57"/>
+      <c r="F50" s="58"/>
     </row>
     <row r="51" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="4">
@@ -2209,11 +2323,11 @@
       <c r="A57" s="56" t="s">
         <v>92</v>
       </c>
-      <c r="B57" s="55"/>
-      <c r="C57" s="55"/>
-      <c r="D57" s="55"/>
-      <c r="E57" s="55"/>
-      <c r="F57" s="55"/>
+      <c r="B57" s="57"/>
+      <c r="C57" s="57"/>
+      <c r="D57" s="57"/>
+      <c r="E57" s="57"/>
+      <c r="F57" s="58"/>
     </row>
     <row r="58" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="4">
@@ -2299,11 +2413,11 @@
       <c r="A62" s="56" t="s">
         <v>102</v>
       </c>
-      <c r="B62" s="55"/>
-      <c r="C62" s="55"/>
-      <c r="D62" s="55"/>
-      <c r="E62" s="55"/>
-      <c r="F62" s="55"/>
+      <c r="B62" s="57"/>
+      <c r="C62" s="57"/>
+      <c r="D62" s="57"/>
+      <c r="E62" s="57"/>
+      <c r="F62" s="58"/>
     </row>
     <row r="63" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="4">
@@ -2403,11 +2517,11 @@
       <c r="A68" s="56" t="s">
         <v>111</v>
       </c>
-      <c r="B68" s="55"/>
-      <c r="C68" s="55"/>
-      <c r="D68" s="55"/>
-      <c r="E68" s="55"/>
-      <c r="F68" s="55"/>
+      <c r="B68" s="57"/>
+      <c r="C68" s="57"/>
+      <c r="D68" s="57"/>
+      <c r="E68" s="57"/>
+      <c r="F68" s="58"/>
     </row>
     <row r="69" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" s="4">
@@ -2511,11 +2625,11 @@
       <c r="A74" s="56" t="s">
         <v>121</v>
       </c>
-      <c r="B74" s="55"/>
-      <c r="C74" s="55"/>
-      <c r="D74" s="55"/>
-      <c r="E74" s="55"/>
-      <c r="F74" s="55"/>
+      <c r="B74" s="57"/>
+      <c r="C74" s="57"/>
+      <c r="D74" s="57"/>
+      <c r="E74" s="57"/>
+      <c r="F74" s="58"/>
     </row>
     <row r="75" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" s="4">
@@ -2621,11 +2735,11 @@
       <c r="A80" s="56" t="s">
         <v>133</v>
       </c>
-      <c r="B80" s="55"/>
-      <c r="C80" s="55"/>
-      <c r="D80" s="55"/>
-      <c r="E80" s="55"/>
-      <c r="F80" s="55"/>
+      <c r="B80" s="57"/>
+      <c r="C80" s="57"/>
+      <c r="D80" s="57"/>
+      <c r="E80" s="57"/>
+      <c r="F80" s="58"/>
     </row>
     <row r="81" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A81" s="4">
@@ -2765,14 +2879,207 @@
         <v>147</v>
       </c>
     </row>
+    <row r="88" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A88" s="60" t="s">
+        <v>148</v>
+      </c>
+      <c r="B88" s="61"/>
+      <c r="C88" s="61"/>
+      <c r="D88" s="61"/>
+      <c r="E88" s="61"/>
+      <c r="F88" s="62"/>
+    </row>
+    <row r="89" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A89" s="4">
+        <v>74</v>
+      </c>
+      <c r="B89" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="C89" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="D89" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E89" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F89" s="8" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A90" s="4">
+        <v>75</v>
+      </c>
+      <c r="B90" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C90" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="D90" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E90" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F90" s="8" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A91" s="4">
+        <v>76</v>
+      </c>
+      <c r="B91" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="C91" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="D91" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E91" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F91" s="8" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A92" s="4">
+        <v>77</v>
+      </c>
+      <c r="B92" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="C92" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="D92" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E92" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F92" s="8" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A93" s="60" t="s">
+        <v>158</v>
+      </c>
+      <c r="B93" s="61"/>
+      <c r="C93" s="61"/>
+      <c r="D93" s="61"/>
+      <c r="E93" s="61"/>
+      <c r="F93" s="62"/>
+    </row>
+    <row r="94" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A94" s="4">
+        <v>78</v>
+      </c>
+      <c r="B94" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="C94" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="D94" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E94" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F94" s="8" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A95" s="4">
+        <v>79</v>
+      </c>
+      <c r="B95" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="C95" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D95" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E95" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F95" s="8" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A96" s="60" t="s">
+        <v>164</v>
+      </c>
+      <c r="B96" s="61"/>
+      <c r="C96" s="61"/>
+      <c r="D96" s="61"/>
+      <c r="E96" s="61"/>
+      <c r="F96" s="62"/>
+    </row>
+    <row r="97" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A97" s="4">
+        <v>80</v>
+      </c>
+      <c r="B97" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="C97" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="D97" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E97" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F97" s="8" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A98" s="4">
+        <v>81</v>
+      </c>
+      <c r="B98" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="C98" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="D98" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E98" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F98" s="8" t="s">
+        <v>169</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A3:F87" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
-  <mergeCells count="13">
+  <mergeCells count="16">
+    <mergeCell ref="A88:F88"/>
+    <mergeCell ref="A93:F93"/>
+    <mergeCell ref="A96:F96"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A68:F68"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A80:F80"/>
     <mergeCell ref="A37:F37"/>
-    <mergeCell ref="A80:F80"/>
     <mergeCell ref="A74:F74"/>
     <mergeCell ref="A17:F17"/>
     <mergeCell ref="A50:F50"/>

</xml_diff>